<commit_message>
feat(documents): 통관SET 컨사이니 블록 확장 + D14=B14 미러 + 연비 H13
- consigneeBlock에 이메일·전화·담당자 추가 (이름/ID/주소/EMAIL/TEL/ATTN 줄바꿈).
  통관SET 구매리스트 B14 + 선적 컨테이너/RORO 인보이스 B9 공용 (전부 wrapText).
- 구매리스트 D14 = `=B14` 수식 (system+karaba 템플릿). 컨사이니 블록 전체를
  Travel Services Invoice F5(=D14)로 미러. ClearanceSetMapping에서 D14 제거.
- 연비 H13 매핑 추가 (nice_spec_fuel_efficiency → 한글/영문등록증 F31 cascade).
  NICE는 fuelCnsmpRt를 NiceApiService에서 이미 매핑하나 미들웨어가 버려
  대부분 공백 → 미들웨어 whitelist 보강 별도 진행.

문서 테스트 40 통과.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/resources/templates/karaba/clearance_set.xlsx
+++ b/resources/templates/karaba/clearance_set.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="378">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="377">
   <si>
     <r>
       <t xml:space="preserve">말소증</t>
@@ -326,11 +326,6 @@
   <si>
     <r>
       <t xml:space="preserve">NAME</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">VIA AUTO</t>
     </r>
   </si>
   <si>
@@ -6135,12 +6130,9 @@
           </r>
         </is>
       </c>
-      <c r="D14" s="118" t="inlineStr">
-        <is>
-          <r>
-            <t xml:space="preserve">VIA AUTO</t>
-          </r>
-        </is>
+      <c r="D14" s="118" t="str">
+        <f>B14</f>
+        <v>0</v>
       </c>
       <c r="E14" s="100"/>
       <c r="F14" s="100"/>
@@ -6827,7 +6819,7 @@
       <c r="C7" s="255"/>
       <c r="D7" s="256"/>
       <c r="E7" s="258" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F7" s="255"/>
       <c r="G7" s="255"/>
@@ -6860,7 +6852,7 @@
       </c>
       <c r="D8" s="255"/>
       <c r="E8" s="260" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F8" s="255"/>
       <c r="G8" s="255"/>
@@ -8454,7 +8446,7 @@
       <c r="C7" s="255"/>
       <c r="D7" s="256"/>
       <c r="E7" s="258" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F7" s="255"/>
       <c r="G7" s="255"/>
@@ -8487,7 +8479,7 @@
       </c>
       <c r="D8" s="255"/>
       <c r="E8" s="260" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="F8" s="255"/>
       <c r="G8" s="255"/>
@@ -10341,7 +10333,7 @@
       </c>
       <c r="D21" s="304"/>
       <c r="E21" s="324" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="F21" s="251"/>
       <c r="G21" s="304"/>
@@ -11250,7 +11242,7 @@
     </row>
     <row r="3" spans="1:10" customHeight="1" ht="18" s="246" customFormat="1">
       <c r="A3" s="346" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="D3" s="263"/>
       <c r="E3" s="229" t="inlineStr">
@@ -12268,7 +12260,7 @@
     </row>
     <row r="3" spans="1:10" customHeight="1" ht="18" s="246" customFormat="1">
       <c r="A3" s="346" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="D3" s="263"/>
       <c r="E3" s="229" t="inlineStr">
@@ -13269,7 +13261,7 @@
     </row>
     <row r="2" spans="1:7" customHeight="1" ht="11.25" s="246" customFormat="1">
       <c r="A2" s="244" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="D2" s="244"/>
     </row>
@@ -13457,7 +13449,7 @@
       </c>
       <c r="B16" s="388"/>
       <c r="C16" s="389" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="D16" s="388"/>
       <c r="E16" s="240" t="inlineStr">
@@ -13468,7 +13460,7 @@
         </is>
       </c>
       <c r="F16" s="390" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="G16" s="388"/>
     </row>
@@ -13482,7 +13474,7 @@
       </c>
       <c r="B17" s="388"/>
       <c r="C17" s="389" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="D17" s="388"/>
       <c r="E17" s="240" t="inlineStr">
@@ -13493,7 +13485,7 @@
         </is>
       </c>
       <c r="F17" s="241" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="G17" s="388"/>
     </row>
@@ -13507,7 +13499,7 @@
       </c>
       <c r="B18" s="388"/>
       <c r="C18" s="389" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="D18" s="388"/>
       <c r="E18" s="240" t="inlineStr">
@@ -13518,7 +13510,7 @@
         </is>
       </c>
       <c r="F18" s="391" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="G18" s="388"/>
     </row>

</xml_diff>